<commit_message>
New figure and intro
</commit_message>
<xml_diff>
--- a/Reply to reviewer comments.xlsx
+++ b/Reply to reviewer comments.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve">Title of the manuscript</t>
   </si>
@@ -25,7 +25,7 @@
   </si>
   <si>
     <t xml:space="preserve">Reviewer comment - 
-mentor</t>
+First reviewer</t>
   </si>
   <si>
     <t xml:space="preserve">Has the comment been addressed? Choose from the dropdown options.</t>
@@ -40,32 +40,41 @@
     <t xml:space="preserve">Major Comments</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;add comment #1&gt;</t>
+    <t xml:space="preserve">Fig1: No panel labels?</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;add comment #2&gt;</t>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">labels added to main figure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is not clear how the MRI regional volumes and biofluid/clinical improve the model stability? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">changed "model stability" to "computation stability" in results to make it clearer that biomarkers were not included in the multilcmm model, only in the secondary analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a paper which needs a table to explain the acronyms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">list of abbreviations added at the top of supplementary</t>
   </si>
   <si>
     <t>.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minor Comments </t>
   </si>
   <si>
     <t xml:space="preserve">Reviewer comment - 
 Second reviewer</t>
   </si>
   <si>
-    <t xml:space="preserve">Fig1: No panel labels?</t>
+    <t xml:space="preserve">Minor Comments </t>
   </si>
   <si>
-    <t>Yes</t>
+    <t xml:space="preserve">I suggest putting Parkinson's disease in the title. I would replace RBDSQ for actual clinical terms and lead with the core finding.</t>
   </si>
   <si>
-    <t xml:space="preserve">It is not clear how the MRI regional volumes and biofluid/clinical improve the model stability? </t>
-  </si>
-  <si>
-    <t xml:space="preserve">changed "model stability" to "computation stability" in results to make it clearer that biomarkers were not included in the multilcmm model, only in the secondary analysis</t>
+    <t xml:space="preserve">New title</t>
   </si>
 </sst>
 </file>
@@ -114,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -128,6 +137,9 @@
     </xf>
     <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -762,11 +774,15 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -792,11 +808,15 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -822,11 +842,15 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
+      <c r="A7" s="6" t="s">
+        <v>12</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -852,9 +876,6 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -882,9 +903,6 @@
       <c r="Z8" s="2"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -912,7 +930,6 @@
       <c r="Z9" s="2"/>
     </row>
     <row r="10">
-      <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -940,9 +957,6 @@
       <c r="Z10" s="2"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -970,9 +984,6 @@
       <c r="Z11" s="2"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
-        <v>7</v>
-      </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -1000,9 +1011,6 @@
       <c r="Z12" s="2"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -1031,7 +1039,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1061,7 +1069,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1091,7 +1099,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1147,11 +1155,19 @@
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
     </row>
-    <row r="18">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+    <row r="18" ht="38.25">
+      <c r="A18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>5</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1176,7 +1192,9 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19">
-      <c r="A19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -1203,19 +1221,11 @@
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" ht="38.25">
-      <c r="A20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>5</v>
-      </c>
+    <row r="20">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1240,9 +1250,7 @@
       <c r="Z20" s="2"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="s">
-        <v>6</v>
-      </c>
+      <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1270,12 +1278,10 @@
       <c r="Z21" s="2"/>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="s">
-        <v>12</v>
+      <c r="A22" s="2" t="s">
+        <v>14</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -1302,15 +1308,11 @@
       <c r="Z22" s="2"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -1364,7 +1366,9 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25">
-      <c r="A25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1392,9 +1396,15 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="A26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>18</v>
+      </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
@@ -1532,9 +1542,7 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1562,9 +1570,7 @@
       <c r="Z31" s="2"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1592,9 +1598,7 @@
       <c r="Z32" s="2"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -28529,174 +28533,6 @@
       <c r="Y994" s="2"/>
       <c r="Z994" s="2"/>
     </row>
-    <row r="995">
-      <c r="A995" s="2"/>
-      <c r="B995" s="2"/>
-      <c r="C995" s="2"/>
-      <c r="D995" s="2"/>
-      <c r="E995" s="2"/>
-      <c r="F995" s="2"/>
-      <c r="G995" s="2"/>
-      <c r="H995" s="2"/>
-      <c r="I995" s="2"/>
-      <c r="J995" s="2"/>
-      <c r="K995" s="2"/>
-      <c r="L995" s="2"/>
-      <c r="M995" s="2"/>
-      <c r="N995" s="2"/>
-      <c r="O995" s="2"/>
-      <c r="P995" s="2"/>
-      <c r="Q995" s="2"/>
-      <c r="R995" s="2"/>
-      <c r="S995" s="2"/>
-      <c r="T995" s="2"/>
-      <c r="U995" s="2"/>
-      <c r="V995" s="2"/>
-      <c r="W995" s="2"/>
-      <c r="X995" s="2"/>
-      <c r="Y995" s="2"/>
-      <c r="Z995" s="2"/>
-    </row>
-    <row r="996">
-      <c r="A996" s="2"/>
-      <c r="B996" s="2"/>
-      <c r="C996" s="2"/>
-      <c r="D996" s="2"/>
-      <c r="E996" s="2"/>
-      <c r="F996" s="2"/>
-      <c r="G996" s="2"/>
-      <c r="H996" s="2"/>
-      <c r="I996" s="2"/>
-      <c r="J996" s="2"/>
-      <c r="K996" s="2"/>
-      <c r="L996" s="2"/>
-      <c r="M996" s="2"/>
-      <c r="N996" s="2"/>
-      <c r="O996" s="2"/>
-      <c r="P996" s="2"/>
-      <c r="Q996" s="2"/>
-      <c r="R996" s="2"/>
-      <c r="S996" s="2"/>
-      <c r="T996" s="2"/>
-      <c r="U996" s="2"/>
-      <c r="V996" s="2"/>
-      <c r="W996" s="2"/>
-      <c r="X996" s="2"/>
-      <c r="Y996" s="2"/>
-      <c r="Z996" s="2"/>
-    </row>
-    <row r="997">
-      <c r="A997" s="2"/>
-      <c r="B997" s="2"/>
-      <c r="C997" s="2"/>
-      <c r="D997" s="2"/>
-      <c r="E997" s="2"/>
-      <c r="F997" s="2"/>
-      <c r="G997" s="2"/>
-      <c r="H997" s="2"/>
-      <c r="I997" s="2"/>
-      <c r="J997" s="2"/>
-      <c r="K997" s="2"/>
-      <c r="L997" s="2"/>
-      <c r="M997" s="2"/>
-      <c r="N997" s="2"/>
-      <c r="O997" s="2"/>
-      <c r="P997" s="2"/>
-      <c r="Q997" s="2"/>
-      <c r="R997" s="2"/>
-      <c r="S997" s="2"/>
-      <c r="T997" s="2"/>
-      <c r="U997" s="2"/>
-      <c r="V997" s="2"/>
-      <c r="W997" s="2"/>
-      <c r="X997" s="2"/>
-      <c r="Y997" s="2"/>
-      <c r="Z997" s="2"/>
-    </row>
-    <row r="998">
-      <c r="A998" s="2"/>
-      <c r="B998" s="2"/>
-      <c r="C998" s="2"/>
-      <c r="D998" s="2"/>
-      <c r="E998" s="2"/>
-      <c r="F998" s="2"/>
-      <c r="G998" s="2"/>
-      <c r="H998" s="2"/>
-      <c r="I998" s="2"/>
-      <c r="J998" s="2"/>
-      <c r="K998" s="2"/>
-      <c r="L998" s="2"/>
-      <c r="M998" s="2"/>
-      <c r="N998" s="2"/>
-      <c r="O998" s="2"/>
-      <c r="P998" s="2"/>
-      <c r="Q998" s="2"/>
-      <c r="R998" s="2"/>
-      <c r="S998" s="2"/>
-      <c r="T998" s="2"/>
-      <c r="U998" s="2"/>
-      <c r="V998" s="2"/>
-      <c r="W998" s="2"/>
-      <c r="X998" s="2"/>
-      <c r="Y998" s="2"/>
-      <c r="Z998" s="2"/>
-    </row>
-    <row r="999">
-      <c r="A999" s="2"/>
-      <c r="B999" s="2"/>
-      <c r="C999" s="2"/>
-      <c r="D999" s="2"/>
-      <c r="E999" s="2"/>
-      <c r="F999" s="2"/>
-      <c r="G999" s="2"/>
-      <c r="H999" s="2"/>
-      <c r="I999" s="2"/>
-      <c r="J999" s="2"/>
-      <c r="K999" s="2"/>
-      <c r="L999" s="2"/>
-      <c r="M999" s="2"/>
-      <c r="N999" s="2"/>
-      <c r="O999" s="2"/>
-      <c r="P999" s="2"/>
-      <c r="Q999" s="2"/>
-      <c r="R999" s="2"/>
-      <c r="S999" s="2"/>
-      <c r="T999" s="2"/>
-      <c r="U999" s="2"/>
-      <c r="V999" s="2"/>
-      <c r="W999" s="2"/>
-      <c r="X999" s="2"/>
-      <c r="Y999" s="2"/>
-      <c r="Z999" s="2"/>
-    </row>
-    <row r="1000">
-      <c r="A1000" s="2"/>
-      <c r="B1000" s="2"/>
-      <c r="C1000" s="2"/>
-      <c r="D1000" s="2"/>
-      <c r="E1000" s="2"/>
-      <c r="F1000" s="2"/>
-      <c r="G1000" s="2"/>
-      <c r="H1000" s="2"/>
-      <c r="I1000" s="2"/>
-      <c r="J1000" s="2"/>
-      <c r="K1000" s="2"/>
-      <c r="L1000" s="2"/>
-      <c r="M1000" s="2"/>
-      <c r="N1000" s="2"/>
-      <c r="O1000" s="2"/>
-      <c r="P1000" s="2"/>
-      <c r="Q1000" s="2"/>
-      <c r="R1000" s="2"/>
-      <c r="S1000" s="2"/>
-      <c r="T1000" s="2"/>
-      <c r="U1000" s="2"/>
-      <c r="V1000" s="2"/>
-      <c r="W1000" s="2"/>
-      <c r="X1000" s="2"/>
-      <c r="Y1000" s="2"/>
-      <c r="Z1000" s="2"/>
-    </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -28705,11 +28541,11 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{00F60027-0054-448F-8001-001B007100CC}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+        <x14:dataValidation xr:uid="{9C48BC84-09E8-4BAC-9B5A-78FF5ED1C396}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Yes,No,Partially"</xm:f>
           </x14:formula1>
-          <xm:sqref>B5:B9 B12:B16 B22:B26 B29:B33</xm:sqref>
+          <xm:sqref>B7:B9 B12:B16 B19:B21 B5:B6 B23:B27</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
MRI Interpretation, Moved Limitations to Supplement, Reviewer Comments
</commit_message>
<xml_diff>
--- a/Reply to reviewer comments.xlsx
+++ b/Reply to reviewer comments.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">Title of the manuscript</t>
   </si>
@@ -61,6 +61,27 @@
     <t xml:space="preserve">list of abbreviations added at the top of supplementary</t>
   </si>
   <si>
+    <t xml:space="preserve">Shap analysis should be in the main text and discussed appropriately. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHAP bar plots and discussion added to main text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Words like seminal, monumental should be used with great concern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This language has been removed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is not clever why variables in box plots are not shown for class 1?</t>
+  </si>
+  <si>
+    <t>Partially</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The caption has been changed to make clearer that only box plots for uncorrected p&lt;0.05 results were plotted, class 1 had no such results</t>
+  </si>
+  <si>
     <t>.</t>
   </si>
   <si>
@@ -75,6 +96,12 @@
   </si>
   <si>
     <t xml:space="preserve">New title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Table 1 has raw statistical console outputs with absurd floating-point precision like 100.00000 and 28.77193. I suggest you round these to standard significant figures.</t>
+  </si>
+  <si>
+    <t>Rounded</t>
   </si>
 </sst>
 </file>
@@ -876,8 +903,15 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8">
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+      <c r="A8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -903,8 +937,15 @@
       <c r="Z8" s="2"/>
     </row>
     <row r="9">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
+      <c r="A9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -930,8 +971,15 @@
       <c r="Z9" s="2"/>
     </row>
     <row r="10">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
+      <c r="A10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1039,7 +1087,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -1069,7 +1117,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1099,7 +1147,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1157,7 +1205,7 @@
     </row>
     <row r="18" ht="38.25">
       <c r="A18" s="3" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>3</v>
@@ -1279,7 +1327,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -1309,7 +1357,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1367,7 +1415,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1397,13 +1445,13 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1430,9 +1478,15 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="A27" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -28540,12 +28594,18 @@
   <headerFooter/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{9C48BC84-09E8-4BAC-9B5A-78FF5ED1C396}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
+        <x14:dataValidation xr:uid="{CBC994AC-6FFD-4348-BB32-62C5F66C7D6A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Yes,No,Partially"</xm:f>
           </x14:formula1>
           <xm:sqref>B7:B9 B12:B16 B19:B21 B5:B6 B23:B27</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{CCE01539-6451-4D9D-A1BC-23AB03A3D5B6}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Yes,No,Partially"</xm:f>
+          </x14:formula1>
+          <xm:sqref>B10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>